<commit_message>
Add option positions to the Positions sheet
The sheet now lists the long NIFTY put and short NIFTY call with quantity, strike, days to expiry and Black-Scholes market value, alongside the equity and FX positions.
</commit_message>
<xml_diff>
--- a/output/risk_report.xlsx
+++ b/output/risk_report.xlsx
@@ -552,11 +552,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -567,6 +571,26 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Asset class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Strike</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Days to expiry</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Market value (INR)</t>
         </is>
       </c>
@@ -577,7 +601,15 @@
           <t>RELIANCE.NS</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -587,7 +619,15 @@
           <t>TCS.NS</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -597,7 +637,15 @@
           <t>HDFCBANK.NS</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -607,7 +655,15 @@
           <t>INFY.NS</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -617,7 +673,15 @@
           <t>ICICIBANK.NS</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -627,7 +691,15 @@
           <t>ITC.NS</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -637,7 +709,15 @@
           <t>LT.NS</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -647,7 +727,15 @@
           <t>SBIN.NS</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" s="3" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -657,8 +745,64 @@
           <t>USDINR=X</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" s="3" t="n">
         <v>1700000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Long NIFTY put (hedge)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>150</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>21973.510234375</v>
+      </c>
+      <c r="E11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>29764.17851506294</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Short NIFTY call</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>-150</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>23094.6076953125</v>
+      </c>
+      <c r="E12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>-36945.74550963157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>